<commit_message>
Log weight through 2026-07-26, fix measure_weight skill
Weight observations appended via the measure_weight skill; iter1.r outputs
(model plot, quarterly summary) regenerated.

Two skill fixes surfaced during use:
- Point at R 4.6.0. The 4.5.2 install has an rlang/ggplot2 mismatch that
  breaks iter1.r.
- Take today's date from `date`, not from conversation context, and only
  warn on a duplicate when the same mass was already logged on the same
  calendar day. The previous wording produced a false duplicate warning.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/martysweight.xlsx
+++ b/inst/extdata/martysweight.xlsx
@@ -45159,6 +45159,699 @@
       </c>
       <c r="G2386"/>
     </row>
+    <row r="2387">
+      <c r="A2387" s="1" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B2387" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2387" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2387" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2387" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2387" t="n">
+        <v>80.7</v>
+      </c>
+      <c r="G2387"/>
+    </row>
+    <row r="2388">
+      <c r="A2388" s="1" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B2388" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2388" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2388" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2388" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2388" t="n">
+        <v>80.7</v>
+      </c>
+      <c r="G2388"/>
+    </row>
+    <row r="2389">
+      <c r="A2389" s="1" t="n">
+        <v>46124</v>
+      </c>
+      <c r="B2389" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2389" t="n">
+        <v>30</v>
+      </c>
+      <c r="D2389" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2389" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2389" t="n">
+        <v>80.7</v>
+      </c>
+      <c r="G2389"/>
+    </row>
+    <row r="2390">
+      <c r="A2390" s="1" t="n">
+        <v>46125</v>
+      </c>
+      <c r="B2390" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2390" t="n">
+        <v>57</v>
+      </c>
+      <c r="D2390" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2390" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2390" t="n">
+        <v>80.3</v>
+      </c>
+      <c r="G2390"/>
+    </row>
+    <row r="2391">
+      <c r="A2391" s="1" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B2391" t="n">
+        <v>11</v>
+      </c>
+      <c r="C2391" t="n">
+        <v>32</v>
+      </c>
+      <c r="D2391" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2391" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2391" t="n">
+        <v>80.3</v>
+      </c>
+      <c r="G2391"/>
+    </row>
+    <row r="2392">
+      <c r="A2392" s="1" t="n">
+        <v>46127</v>
+      </c>
+      <c r="B2392" t="n">
+        <v>9</v>
+      </c>
+      <c r="C2392" t="n">
+        <v>13</v>
+      </c>
+      <c r="D2392" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2392" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2392" t="n">
+        <v>80.2</v>
+      </c>
+      <c r="G2392"/>
+    </row>
+    <row r="2393">
+      <c r="A2393" s="1" t="n">
+        <v>46130</v>
+      </c>
+      <c r="B2393" t="n">
+        <v>9</v>
+      </c>
+      <c r="C2393" t="n">
+        <v>9</v>
+      </c>
+      <c r="D2393" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2393" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2393" t="n">
+        <v>80</v>
+      </c>
+      <c r="G2393"/>
+    </row>
+    <row r="2394">
+      <c r="A2394" s="1" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B2394" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2394" t="n">
+        <v>30</v>
+      </c>
+      <c r="D2394" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2394" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2394" t="n">
+        <v>80.8</v>
+      </c>
+      <c r="G2394"/>
+    </row>
+    <row r="2395">
+      <c r="A2395" s="1" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B2395" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2395" t="n">
+        <v>45</v>
+      </c>
+      <c r="D2395" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2395" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2395" t="n">
+        <v>80.3</v>
+      </c>
+      <c r="G2395"/>
+    </row>
+    <row r="2396">
+      <c r="A2396" s="1" t="n">
+        <v>46134</v>
+      </c>
+      <c r="B2396" t="n">
+        <v>11</v>
+      </c>
+      <c r="C2396" t="n">
+        <v>7</v>
+      </c>
+      <c r="D2396" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2396" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2396" t="n">
+        <v>80.3</v>
+      </c>
+      <c r="G2396"/>
+    </row>
+    <row r="2397">
+      <c r="A2397" s="1" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B2397" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2397" t="n">
+        <v>21</v>
+      </c>
+      <c r="D2397" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2397" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2397" t="n">
+        <v>79.9</v>
+      </c>
+      <c r="G2397"/>
+    </row>
+    <row r="2398">
+      <c r="A2398" s="1" t="n">
+        <v>46136</v>
+      </c>
+      <c r="B2398" t="n">
+        <v>11</v>
+      </c>
+      <c r="C2398" t="n">
+        <v>21</v>
+      </c>
+      <c r="D2398" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2398" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2398" t="n">
+        <v>79.9</v>
+      </c>
+      <c r="G2398"/>
+    </row>
+    <row r="2399">
+      <c r="A2399" s="1" t="n">
+        <v>46138</v>
+      </c>
+      <c r="B2399" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2399" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2399" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2399" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2399" t="n">
+        <v>80.4</v>
+      </c>
+      <c r="G2399"/>
+    </row>
+    <row r="2400">
+      <c r="A2400" s="1" t="n">
+        <v>46139</v>
+      </c>
+      <c r="B2400" t="n">
+        <v>11</v>
+      </c>
+      <c r="C2400" t="n">
+        <v>24</v>
+      </c>
+      <c r="D2400" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2400" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2400" t="n">
+        <v>80.4</v>
+      </c>
+      <c r="G2400"/>
+    </row>
+    <row r="2401">
+      <c r="A2401" s="1" t="n">
+        <v>46140</v>
+      </c>
+      <c r="B2401" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2401" t="n">
+        <v>42</v>
+      </c>
+      <c r="D2401" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2401" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2401" t="n">
+        <v>80.4</v>
+      </c>
+      <c r="G2401"/>
+    </row>
+    <row r="2402">
+      <c r="A2402" s="1" t="n">
+        <v>46141</v>
+      </c>
+      <c r="B2402" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2402" t="n">
+        <v>42</v>
+      </c>
+      <c r="D2402" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2402" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2402" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="G2402"/>
+    </row>
+    <row r="2403">
+      <c r="A2403" s="1" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B2403" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2403" t="n">
+        <v>32</v>
+      </c>
+      <c r="D2403" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2403" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2403" t="n">
+        <v>80.4</v>
+      </c>
+      <c r="G2403"/>
+    </row>
+    <row r="2404">
+      <c r="A2404" s="1" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B2404" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2404" t="n">
+        <v>32</v>
+      </c>
+      <c r="D2404" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2404" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2404" t="n">
+        <v>80.4</v>
+      </c>
+      <c r="G2404"/>
+    </row>
+    <row r="2405">
+      <c r="A2405" s="1" t="n">
+        <v>46148</v>
+      </c>
+      <c r="B2405" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2405" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2405" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2405" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2405" t="n">
+        <v>79.9</v>
+      </c>
+      <c r="G2405"/>
+    </row>
+    <row r="2406">
+      <c r="A2406" s="1" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B2406" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2406" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2406" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2406" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2406" t="n">
+        <v>79.7</v>
+      </c>
+      <c r="G2406"/>
+    </row>
+    <row r="2407">
+      <c r="A2407" s="1" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B2407" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2407" t="n">
+        <v>47</v>
+      </c>
+      <c r="D2407" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2407" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2407" t="n">
+        <v>80</v>
+      </c>
+      <c r="G2407"/>
+    </row>
+    <row r="2408">
+      <c r="A2408" s="1" t="n">
+        <v>46160</v>
+      </c>
+      <c r="B2408" t="n">
+        <v>9</v>
+      </c>
+      <c r="C2408" t="n">
+        <v>50</v>
+      </c>
+      <c r="D2408" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2408" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2408" t="n">
+        <v>79.9</v>
+      </c>
+      <c r="G2408"/>
+    </row>
+    <row r="2409">
+      <c r="A2409" s="1" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B2409" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2409" t="n">
+        <v>59</v>
+      </c>
+      <c r="D2409" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2409" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2409" t="n">
+        <v>79.2</v>
+      </c>
+      <c r="G2409"/>
+    </row>
+    <row r="2410">
+      <c r="A2410" s="1" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B2410" t="n">
+        <v>6</v>
+      </c>
+      <c r="C2410" t="n">
+        <v>47</v>
+      </c>
+      <c r="D2410" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2410" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2410" t="n">
+        <v>79.2</v>
+      </c>
+      <c r="G2410"/>
+    </row>
+    <row r="2411">
+      <c r="A2411" s="1" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B2411" t="n">
+        <v>16</v>
+      </c>
+      <c r="C2411" t="n">
+        <v>4</v>
+      </c>
+      <c r="D2411" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2411" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2411" t="n">
+        <v>79.6</v>
+      </c>
+      <c r="G2411"/>
+    </row>
+    <row r="2412">
+      <c r="A2412" s="1" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B2412" t="n">
+        <v>9</v>
+      </c>
+      <c r="C2412" t="n">
+        <v>22</v>
+      </c>
+      <c r="D2412" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2412" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2412" t="n">
+        <v>79.2</v>
+      </c>
+      <c r="G2412"/>
+    </row>
+    <row r="2413">
+      <c r="A2413" s="1" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B2413" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2413" t="n">
+        <v>27</v>
+      </c>
+      <c r="D2413" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2413" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2413" t="n">
+        <v>79.1</v>
+      </c>
+      <c r="G2413"/>
+    </row>
+    <row r="2414">
+      <c r="A2414" s="1" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B2414" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2414" t="n">
+        <v>53</v>
+      </c>
+      <c r="D2414" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2414" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2414" t="n">
+        <v>78.9</v>
+      </c>
+      <c r="G2414"/>
+    </row>
+    <row r="2415">
+      <c r="A2415" s="1" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B2415" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2415" t="n">
+        <v>33</v>
+      </c>
+      <c r="D2415" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2415" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2415" t="n">
+        <v>79.6</v>
+      </c>
+      <c r="G2415"/>
+    </row>
+    <row r="2416">
+      <c r="A2416" s="1" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B2416" t="n">
+        <v>9</v>
+      </c>
+      <c r="C2416" t="n">
+        <v>48</v>
+      </c>
+      <c r="D2416" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2416" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2416" t="n">
+        <v>79.3</v>
+      </c>
+      <c r="G2416"/>
+    </row>
+    <row r="2417">
+      <c r="A2417" s="1" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B2417" t="n">
+        <v>11</v>
+      </c>
+      <c r="C2417" t="n">
+        <v>32</v>
+      </c>
+      <c r="D2417" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2417" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2417" t="n">
+        <v>78.8</v>
+      </c>
+      <c r="G2417"/>
+    </row>
+    <row r="2418">
+      <c r="A2418" s="1" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B2418" t="n">
+        <v>12</v>
+      </c>
+      <c r="C2418" t="n">
+        <v>55</v>
+      </c>
+      <c r="D2418" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2418" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2418" t="n">
+        <v>79</v>
+      </c>
+      <c r="G2418"/>
+    </row>
+    <row r="2419">
+      <c r="A2419" s="1" t="n">
+        <v>46229</v>
+      </c>
+      <c r="B2419" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2419" t="n">
+        <v>59</v>
+      </c>
+      <c r="D2419" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2419" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2419" t="n">
+        <v>79.1</v>
+      </c>
+      <c r="G2419"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>